<commit_message>
Regenerate documents and decks, add Technology Architecture v2
- Update 9 generators (demo scripts, setup/creation guides, glossary
  Excel, architecture and demo overview decks, carriers, governance)
- Regenerate all 38 Word/Excel documents and both PPTX decks
- Add MCG_Technology_Architecture_v2.pptx

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/MCG_Business_Glossary.xlsx
+++ b/documents/MCG_Business_Glossary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="195">
   <si>
     <t>Category</t>
   </si>
@@ -117,9 +117,6 @@
     <t>#1 — Phantom Inventory, #7 — Compliance Gap</t>
   </si>
   <si>
-    <t>Supply Chain Health, Compliance Readiness</t>
-  </si>
-  <si>
     <t>bronze.warehouse_events (event_type='RECEIVE')</t>
   </si>
   <si>
@@ -138,9 +135,6 @@
     <t>#7 — Compliance Traceability Gap</t>
   </si>
   <si>
-    <t>Compliance Readiness</t>
-  </si>
-  <si>
     <t>silver.inventory_reconciled (lot_number field)</t>
   </si>
   <si>
@@ -165,10 +159,10 @@
     <t>#6 — Carrier Data Black Hole</t>
   </si>
   <si>
-    <t>Customer Delivery Experience, Last Mile Performance</t>
-  </si>
-  <si>
-    <t>gold.customer_delivery_experience, gold.last_mile_performance</t>
+    <t>Last Mile Performance</t>
+  </si>
+  <si>
+    <t>gold.last_mile_performance</t>
   </si>
   <si>
     <t>Lisa Park (Head of Customer Experience)</t>
@@ -189,9 +183,6 @@
     <t>#2 — Address Catastrophe, #6 — Carrier Black Hole</t>
   </si>
   <si>
-    <t>Last Mile Performance</t>
-  </si>
-  <si>
     <t>gold.last_mile_performance (sla_met field)</t>
   </si>
   <si>
@@ -210,10 +201,7 @@
     <t>A temperature violation where a refrigerated or frozen shipment exceeds its maximum allowable temperature threshold for a specified duration. MCG thresholds: &gt;8°C for &gt;30 min (fresh produce), &gt;8°C for &gt;15 min (dairy), any reading above threshold (frozen).</t>
   </si>
   <si>
-    <t>Cold Chain Compliance</t>
-  </si>
-  <si>
-    <t>gold.cold_chain_compliance, silver.iot_normalized</t>
+    <t>silver.iot_normalized</t>
   </si>
   <si>
     <t>Thomas Brennan (VP Supply Chain)</t>
@@ -234,12 +222,6 @@
     <t>#2 — Address Catastrophe</t>
   </si>
   <si>
-    <t>Customer Delivery Experience</t>
-  </si>
-  <si>
-    <t>gold.customer_delivery_experience</t>
-  </si>
-  <si>
     <t>MCG-POL-020</t>
   </si>
   <si>
@@ -252,7 +234,7 @@
     <t>The requirement that refrigerated transport vehicles must reach target temperature before loading cold chain products. Ensures the cold chain is maintained from warehouse to destination without initial temperature spikes.</t>
   </si>
   <si>
-    <t>gold.cold_chain_compliance (pre_cool_compliant field)</t>
+    <t>silver.iot_normalized (pre_cool_compliant field)</t>
   </si>
   <si>
     <t>Failed pre-cool is the #1 predictor of spoilage on long routes</t>
@@ -315,7 +297,7 @@
     <t>All nightmares affect Trust Score</t>
   </si>
   <si>
-    <t>All 8 data products</t>
+    <t>Supply Chain Health, Last Mile Performance</t>
   </si>
   <si>
     <t>Applied to gold.* tables via Qlik Data Products</t>
@@ -378,7 +360,7 @@
     <t>Netherlands Food and Consumer Product Safety Authority (Nederlandse Voedsel- en Warenautoriteit). The Dutch regulatory body responsible for food safety enforcement. MCG's Rotterdam DC is subject to NVWA inspections.</t>
   </si>
   <si>
-    <t>gold.compliance_readiness</t>
+    <t>silver.inventory_reconciled</t>
   </si>
   <si>
     <t>COMP-2025-NVWA, MCG-POL-007</t>
@@ -408,10 +390,7 @@
     <t>#3 — Product Master Mess, #7 — Compliance Gap</t>
   </si>
   <si>
-    <t>Product Master 360, Compliance Readiness</t>
-  </si>
-  <si>
-    <t>silver.suppliers_deduped, gold.product_master_360</t>
+    <t>silver.suppliers_deduped, silver.products_harmonized</t>
   </si>
   <si>
     <t>Thomas Berger (Product Data Manager)</t>
@@ -432,10 +411,7 @@
     <t>#3 — Product Master Mess</t>
   </si>
   <si>
-    <t>Product Master 360</t>
-  </si>
-  <si>
-    <t>silver.products_harmonized, gold.product_master_360</t>
+    <t>silver.products_harmonized</t>
   </si>
   <si>
     <t>Invalid GTINs block EDI orders and retail compliance</t>
@@ -504,7 +480,7 @@
     <t>N/A — Gold is the outcome of fixing nightmares</t>
   </si>
   <si>
-    <t>gold.supply_chain_health, gold.last_mile_performance, gold.cold_chain_compliance, gold.product_master_360, gold.customer_delivery_experience, gold.compliance_readiness, gold.operational_cost_impact, gold.order_timeline</t>
+    <t>gold.supply_chain_health, gold.last_mile_performance</t>
   </si>
   <si>
     <t>Single source of truth for all analytics, AI, and external consumers</t>
@@ -514,9 +490,6 @@
   </si>
   <si>
     <t>MCG's unified shipment status vocabulary that normalizes 6 carriers × 6 languages into a single lifecycle: LABEL_CREATED → PICKED_UP → IN_TRANSIT → OUT_FOR_DELIVERY → DELIVERED (or FAILED/RETURNED).</t>
-  </si>
-  <si>
-    <t>Last Mile Performance, Customer Delivery Experience</t>
   </si>
   <si>
     <t>silver.shipments_canonical (status_canonical field)</t>
@@ -1302,19 +1275,19 @@
         <v>33</v>
       </c>
       <c r="F5" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>35</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1322,671 +1295,671 @@
         <v>10</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="E7" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="H7" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="I7" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="J7" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="6" t="s">
+      <c r="F8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="10" t="s">
+      <c r="I9" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9" s="10" t="s">
+      <c r="J9" s="10" t="s">
         <v>65</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="H12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="I12" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="J12" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="J14" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J16" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F17" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="G17" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>43</v>
-      </c>
       <c r="I17" s="10" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="C18" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="I18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="J18" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B19" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="J19" s="10" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>139</v>
+        <v>15</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="H20" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>139</v>
+        <v>94</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>154</v>
-      </c>
       <c r="C23" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="J23" s="10" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="24" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="25" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>167</v>
+        <v>48</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="J25" s="10" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2012,16 +1985,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -2032,86 +2005,86 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" s="7">
         <v>5</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B4" s="3">
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B5" s="7">
         <v>5</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B7" s="21">
         <v>25</v>
@@ -2120,7 +2093,7 @@
         <v>12</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="E7" s="21" t="s">
         <v>12</v>
@@ -2147,22 +2120,22 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2179,7 +2152,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>17</v>
@@ -2199,7 +2172,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>17</v>
@@ -2219,7 +2192,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>17</v>
@@ -2239,7 +2212,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>17</v>
@@ -2247,10 +2220,10 @@
     </row>
     <row r="6" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>12</v>
@@ -2259,410 +2232,410 @@
         <v>10</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>